<commit_message>
used some recommendations from the group today. and working on something
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shawn\Downloads\UNR\CS 425\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2559638D-1CC0-4437-AF7B-E120DF8CAAC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41EE2C15-A753-484E-8FFD-9EA70EEC5875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5064" yWindow="5880" windowWidth="15852" windowHeight="7524" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>
@@ -418,16 +418,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="26.21875" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" customWidth="1"/>
-    <col min="6" max="7" width="28.6640625" customWidth="1"/>
-    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+    <col min="2" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" customWidth="1"/>
+    <col min="6" max="7" width="28.7109375" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -453,7 +453,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <f t="shared" ref="A2:A3" si="0">ROW()-2</f>
         <v>0</v>
@@ -462,10 +462,10 @@
         <v>14</v>
       </c>
       <c r="C2">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -481,7 +481,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -490,10 +490,10 @@
         <v>15</v>
       </c>
       <c r="C3">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="D3">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -509,7 +509,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>ROW()-2</f>
         <v>2</v>
@@ -518,10 +518,10 @@
         <v>16</v>
       </c>
       <c r="C4">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="D4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4">
         <v>6</v>
@@ -537,7 +537,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <f>ROW()-2</f>
         <v>3</v>
@@ -546,10 +546,10 @@
         <v>17</v>
       </c>
       <c r="C5">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="D5">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>10</v>
@@ -565,7 +565,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <f>ROW()-2</f>
         <v>4</v>
@@ -574,10 +574,10 @@
         <v>18</v>
       </c>
       <c r="C6">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -602,13 +602,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6544C360-8E1E-43B6-9EF8-C40FD311EE72}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.77734375" customWidth="1"/>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -616,7 +616,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -625,7 +625,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A6" si="0">ROW()-2</f>
         <v>1</v>
@@ -634,7 +634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -643,7 +643,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -652,7 +652,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>

</xml_diff>

<commit_message>
enemy now gets destroyed
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41EE2C15-A753-484E-8FFD-9EA70EEC5875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B184A8-63F7-427F-B753-FA2669AC51D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added fade out for the interactable text and changed enemy names
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B184A8-63F7-427F-B753-FA2669AC51D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C35CB39-07B8-43E3-A6DB-6C51EE36A4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -81,19 +81,19 @@
     <t>Attack5</t>
   </si>
   <si>
-    <t>An Unremarkable Zombie</t>
-  </si>
-  <si>
-    <t>Teen Zombie</t>
-  </si>
-  <si>
-    <t>Girl Zombie</t>
-  </si>
-  <si>
-    <t>Midlife Crisis Zombie</t>
-  </si>
-  <si>
-    <t>Loser Zombie</t>
+    <t>The Substitute Teacher</t>
+  </si>
+  <si>
+    <t>The Class President</t>
+  </si>
+  <si>
+    <t>The Mall Security Guard</t>
+  </si>
+  <si>
+    <t>The Divorced Salesman</t>
+  </si>
+  <si>
+    <t>The Taxi Driver</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
added a results panel after winning battle and added one boss with a unique mechanic
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C35CB39-07B8-43E3-A6DB-6C51EE36A4CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8E9622-50F2-4F4C-B832-D49A9E8D41A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>
@@ -418,16 +418,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="26.28515625" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" customWidth="1"/>
-    <col min="6" max="7" width="28.7109375" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" customWidth="1"/>
+    <col min="2" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" customWidth="1"/>
+    <col min="6" max="7" width="28.6640625" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -453,7 +453,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A3" si="0">ROW()-2</f>
         <v>0</v>
@@ -481,7 +481,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -509,7 +509,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>ROW()-2</f>
         <v>2</v>
@@ -537,7 +537,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>ROW()-2</f>
         <v>3</v>
@@ -565,7 +565,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>ROW()-2</f>
         <v>4</v>
@@ -574,13 +574,13 @@
         <v>18</v>
       </c>
       <c r="C6">
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="D6">
         <v>25</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6">
         <v>4</v>
@@ -602,13 +602,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6544C360-8E1E-43B6-9EF8-C40FD311EE72}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -616,7 +616,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -625,7 +625,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" ref="A3:A6" si="0">ROW()-2</f>
         <v>1</v>
@@ -634,7 +634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -643,7 +643,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -652,7 +652,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>

</xml_diff>

<commit_message>
added a final boss in level_2
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes\CS 425\Unity Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8E9622-50F2-4F4C-B832-D49A9E8D41A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA99B2A1-23AA-490F-BD65-EDA9FE7872A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>ID</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t>The Taxi Driver</t>
+  </si>
+  <si>
+    <t>Isaac</t>
+  </si>
+  <si>
+    <t>Attack6</t>
   </si>
 </sst>
 </file>
@@ -417,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="19.6640625" customWidth="1"/>
@@ -590,6 +596,33 @@
         <v>Attack5</v>
       </c>
       <c r="H6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <f>ROW() - 2</f>
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7">
+        <v>210</v>
+      </c>
+      <c r="D7">
+        <v>35</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added a miniboss and interactables for level_1_hospital
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes\CS 425\Unity Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA99B2A1-23AA-490F-BD65-EDA9FE7872A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD20E003-CBE5-4C31-84F3-2A361ED2DF58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>ID</t>
   </si>
@@ -100,6 +100,12 @@
   </si>
   <si>
     <t>Attack6</t>
+  </si>
+  <si>
+    <t>Trevor</t>
+  </si>
+  <si>
+    <t>Attack7</t>
   </si>
 </sst>
 </file>
@@ -423,17 +429,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" customWidth="1"/>
-    <col min="6" max="7" width="28.6640625" customWidth="1"/>
-    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+    <col min="2" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" customWidth="1"/>
+    <col min="6" max="7" width="28.7109375" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -459,7 +465,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <f t="shared" ref="A2:A3" si="0">ROW()-2</f>
         <v>0</v>
@@ -487,7 +493,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -515,7 +521,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>ROW()-2</f>
         <v>2</v>
@@ -543,7 +549,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <f>ROW()-2</f>
         <v>3</v>
@@ -571,7 +577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <f>ROW()-2</f>
         <v>4</v>
@@ -599,7 +605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <f>ROW() - 2</f>
         <v>5</v>
@@ -623,6 +629,33 @@
         <v>20</v>
       </c>
       <c r="H7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <f xml:space="preserve"> ROW() - 2</f>
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8">
+        <v>165</v>
+      </c>
+      <c r="D8">
+        <v>28</v>
+      </c>
+      <c r="E8">
+        <v>11</v>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+      <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8">
         <v>5</v>
       </c>
     </row>
@@ -635,13 +668,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6544C360-8E1E-43B6-9EF8-C40FD311EE72}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -649,7 +682,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -658,7 +691,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A6" si="0">ROW()-2</f>
         <v>1</v>
@@ -667,7 +700,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -676,7 +709,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -685,7 +718,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>

</xml_diff>

<commit_message>
added separate music for the bosses and minibosses in battle
only regular enemies keep the same battle music track we have
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD20E003-CBE5-4C31-84F3-2A361ED2DF58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FAED82-3026-4C45-8D8C-6992197BA006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5370" yWindow="3555" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>
@@ -477,7 +477,7 @@
         <v>100</v>
       </c>
       <c r="D2">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -502,7 +502,7 @@
         <v>15</v>
       </c>
       <c r="C3">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D3">
         <v>15</v>
@@ -530,7 +530,7 @@
         <v>16</v>
       </c>
       <c r="C4">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -586,7 +586,7 @@
         <v>18</v>
       </c>
       <c r="C6">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D6">
         <v>25</v>
@@ -641,7 +641,7 @@
         <v>21</v>
       </c>
       <c r="C8">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="D8">
         <v>28</v>

</xml_diff>

<commit_message>
new zombie sprites are now set with enemy id
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smast\Documents\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FAED82-3026-4C45-8D8C-6992197BA006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1784284-5C5D-420E-ADFD-4763A88488B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5370" yWindow="3555" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>ID</t>
   </si>
@@ -106,6 +106,48 @@
   </si>
   <si>
     <t>Attack7</t>
+  </si>
+  <si>
+    <t>Attack8</t>
+  </si>
+  <si>
+    <t>Undead Criminal</t>
+  </si>
+  <si>
+    <t>The Lumberjack</t>
+  </si>
+  <si>
+    <t>The Dock Worker</t>
+  </si>
+  <si>
+    <t>The Demolition Man</t>
+  </si>
+  <si>
+    <t>Hazmat Zombie</t>
+  </si>
+  <si>
+    <t>Heavy Weapons Guy</t>
+  </si>
+  <si>
+    <t>The Mysterious Wandere</t>
+  </si>
+  <si>
+    <t>Undead Scientist</t>
+  </si>
+  <si>
+    <t>The Plumber</t>
+  </si>
+  <si>
+    <t>Undead Tourist</t>
+  </si>
+  <si>
+    <t>Undead Soldier</t>
+  </si>
+  <si>
+    <t>The Security Guard</t>
+  </si>
+  <si>
+    <t>Attack 8</t>
   </si>
 </sst>
 </file>
@@ -429,17 +471,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="26.28515625" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" customWidth="1"/>
-    <col min="6" max="7" width="28.7109375" customWidth="1"/>
-    <col min="8" max="8" width="24.85546875" customWidth="1"/>
+    <col min="2" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" customWidth="1"/>
+    <col min="6" max="7" width="28.6640625" customWidth="1"/>
+    <col min="8" max="8" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -465,7 +507,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A3" si="0">ROW()-2</f>
         <v>0</v>
@@ -493,7 +535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -521,7 +563,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>ROW()-2</f>
         <v>2</v>
@@ -549,7 +591,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>ROW()-2</f>
         <v>3</v>
@@ -577,7 +619,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>ROW()-2</f>
         <v>4</v>
@@ -605,7 +647,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>ROW() - 2</f>
         <v>5</v>
@@ -632,7 +674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
         <f xml:space="preserve"> ROW() - 2</f>
         <v>6</v>
@@ -657,6 +699,282 @@
       </c>
       <c r="H8">
         <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9">
+        <v>75</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+      <c r="G9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10">
+        <v>75</v>
+      </c>
+      <c r="D10">
+        <v>10</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+      <c r="F10">
+        <v>7</v>
+      </c>
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11">
+        <v>75</v>
+      </c>
+      <c r="D11">
+        <v>10</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>7</v>
+      </c>
+      <c r="G11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>75</v>
+      </c>
+      <c r="D12">
+        <v>10</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>7</v>
+      </c>
+      <c r="G12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13">
+        <v>75</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>7</v>
+      </c>
+      <c r="G13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14">
+        <v>75</v>
+      </c>
+      <c r="D14">
+        <v>10</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>7</v>
+      </c>
+      <c r="G14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15">
+        <v>75</v>
+      </c>
+      <c r="D15">
+        <v>10</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>7</v>
+      </c>
+      <c r="G15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16">
+        <v>75</v>
+      </c>
+      <c r="D16">
+        <v>10</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>7</v>
+      </c>
+      <c r="G16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17">
+        <v>75</v>
+      </c>
+      <c r="D17">
+        <v>10</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <v>7</v>
+      </c>
+      <c r="G17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18">
+        <v>75</v>
+      </c>
+      <c r="D18">
+        <v>10</v>
+      </c>
+      <c r="E18">
+        <v>2</v>
+      </c>
+      <c r="F18">
+        <v>7</v>
+      </c>
+      <c r="G18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19">
+        <v>75</v>
+      </c>
+      <c r="D19">
+        <v>10</v>
+      </c>
+      <c r="E19">
+        <v>2</v>
+      </c>
+      <c r="F19">
+        <v>7</v>
+      </c>
+      <c r="G19" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20">
+        <v>75</v>
+      </c>
+      <c r="D20">
+        <v>10</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <v>7</v>
+      </c>
+      <c r="G20" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -668,13 +986,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6544C360-8E1E-43B6-9EF8-C40FD311EE72}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -682,7 +1000,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -691,7 +1009,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" ref="A3:A6" si="0">ROW()-2</f>
         <v>1</v>
@@ -700,7 +1018,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -709,7 +1027,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -718,7 +1036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>

</xml_diff>

<commit_message>
added more sfx for the new enemies
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
+++ b/Assets/StreamingAssets/Excel/Value/EnemyValue.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smast\Documents\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNR Classes and Files\CS 425 - Software Engineering\Senior Projects - Game\CS425-426\Assets\StreamingAssets\Excel\Value\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1784284-5C5D-420E-ADFD-4763A88488B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B907B9D8-0BDB-42FC-AE71-03D5ACC2B787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1260" yWindow="1380" windowWidth="21600" windowHeight="12150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyValue" sheetId="1" r:id="rId1"/>
@@ -472,16 +472,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="19.6640625" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" customWidth="1"/>
-    <col min="5" max="5" width="9.5546875" customWidth="1"/>
-    <col min="6" max="7" width="28.6640625" customWidth="1"/>
-    <col min="8" max="8" width="24.88671875" customWidth="1"/>
+    <col min="2" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" customWidth="1"/>
+    <col min="6" max="7" width="28.7109375" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,7 +507,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <f t="shared" ref="A2:A3" si="0">ROW()-2</f>
         <v>0</v>
@@ -535,7 +535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -563,7 +563,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>ROW()-2</f>
         <v>2</v>
@@ -591,7 +591,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <f>ROW()-2</f>
         <v>3</v>
@@ -619,7 +619,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <f>ROW()-2</f>
         <v>4</v>
@@ -647,7 +647,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <f>ROW() - 2</f>
         <v>5</v>
@@ -659,7 +659,7 @@
         <v>210</v>
       </c>
       <c r="D7">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -674,7 +674,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <f xml:space="preserve"> ROW() - 2</f>
         <v>6</v>
@@ -701,7 +701,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -709,10 +709,10 @@
         <v>24</v>
       </c>
       <c r="C9">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -724,7 +724,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -732,10 +732,10 @@
         <v>25</v>
       </c>
       <c r="C10">
-        <v>75</v>
+        <v>115</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E10">
         <v>2</v>
@@ -747,7 +747,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -755,10 +755,10 @@
         <v>26</v>
       </c>
       <c r="C11">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="D11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E11">
         <v>2</v>
@@ -770,7 +770,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -778,10 +778,10 @@
         <v>27</v>
       </c>
       <c r="C12">
-        <v>75</v>
+        <v>115</v>
       </c>
       <c r="D12">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -793,7 +793,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -801,10 +801,10 @@
         <v>28</v>
       </c>
       <c r="C13">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D13">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -816,7 +816,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -824,10 +824,10 @@
         <v>29</v>
       </c>
       <c r="C14">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="D14">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -839,7 +839,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -847,10 +847,10 @@
         <v>30</v>
       </c>
       <c r="C15">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="D15">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E15">
         <v>2</v>
@@ -862,7 +862,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -870,10 +870,10 @@
         <v>31</v>
       </c>
       <c r="C16">
-        <v>75</v>
+        <v>115</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E16">
         <v>2</v>
@@ -885,7 +885,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -893,10 +893,10 @@
         <v>32</v>
       </c>
       <c r="C17">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D17">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E17">
         <v>2</v>
@@ -908,7 +908,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -916,10 +916,10 @@
         <v>35</v>
       </c>
       <c r="C18">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E18">
         <v>2</v>
@@ -931,7 +931,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -939,10 +939,10 @@
         <v>33</v>
       </c>
       <c r="C19">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D19">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E19">
         <v>2</v>
@@ -954,7 +954,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -962,10 +962,10 @@
         <v>34</v>
       </c>
       <c r="C20">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="D20">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -986,13 +986,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6544C360-8E1E-43B6-9EF8-C40FD311EE72}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <f>ROW()-2</f>
         <v>0</v>
@@ -1009,7 +1009,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" ref="A3:A6" si="0">ROW()-2</f>
         <v>1</v>
@@ -1018,7 +1018,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -1027,7 +1027,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1036,7 +1036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>

</xml_diff>